<commit_message>
Admin panel enhancements and navigation updates
</commit_message>
<xml_diff>
--- a/dataset/Global Income Distribution Dataset.xlsx
+++ b/dataset/Global Income Distribution Dataset.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\onkar\Desktop\infosys springboard virtual internship (1)\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\onkar\Desktop\infosys springboard virtual internship (1)\dataset\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0479F5D-9732-4775-8C39-A33631CFEBA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D4BBF67-9E27-4897-8872-AC6A1861981C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{BCCAE708-985E-4D9B-804A-5FC41DCE8055}"/>
   </bookViews>

</xml_diff>